<commit_message>
generate potongan gaji Excel and refactor phase 4 logic with dynamic headers, helpers, and additional metadata
</commit_message>
<xml_diff>
--- a/excel_template/potongan_gaji_template.xlsx
+++ b/excel_template/potongan_gaji_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\python\penggajian-kafka\excel_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7D2E633B-4904-4CB9-95B1-2F54025BF96F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1587F8BE-54AF-4724-8AB8-4F5568C25378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{F5B233D3-6CBB-4568-8740-04019DC61ED5}"/>
+    <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{F5B233D3-6CBB-4568-8740-04019DC61ED5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>PEMERINTAH KABUPATEN BANYUMAS</t>
   </si>
@@ -61,18 +61,6 @@
   </si>
   <si>
     <t>GAJI</t>
-  </si>
-  <si>
-    <t>POTONGAN</t>
-  </si>
-  <si>
-    <t>JUMLAH POTONGAN</t>
-  </si>
-  <si>
-    <t>GAJI BERSIH</t>
-  </si>
-  <si>
-    <t>(belum ada data)</t>
   </si>
   <si>
     <t>BIDANG</t>
@@ -145,26 +133,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -479,136 +462,96 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9AD43C1-B394-4113-B069-C80E324F2872}">
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="34.90625" customWidth="1"/>
-    <col min="3" max="3" width="15.6328125" customWidth="1"/>
-    <col min="4" max="4" width="20.6328125" customWidth="1"/>
-    <col min="5" max="7" width="17.54296875" customWidth="1"/>
+    <col min="2" max="2" width="34.88671875" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="1" t="s">
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+    </row>
+    <row r="4" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+    </row>
+    <row r="5" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="5" t="s">
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A6:G6"/>
+  <mergeCells count="4">
     <mergeCell ref="A9:A10"/>
     <mergeCell ref="B9:B10"/>
     <mergeCell ref="C9:C10"/>
     <mergeCell ref="D9:D10"/>
-    <mergeCell ref="F9:F10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>